<commit_message>
Sync situação updates from source spreadsheets (8 FC + 3 PO changes)
Most changes reflect new exonerações; Paulo Egidio Alves de Oliveira
moved to FIM DE FILA in FC and EXONERAÇÃO in PO.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Aprovados PO.xlsx
+++ b/Aprovados PO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brunorvmaciel/claude-projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE4631D-D539-FB45-865B-6ED30A421CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F1CD0FF-99D9-2946-B2E0-1E1A35327BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="1100" windowWidth="27840" windowHeight="15380" xr2:uid="{480248C0-AF05-6948-87A4-21BF4011A9C0}"/>
   </bookViews>
@@ -261,7 +261,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -291,9 +291,20 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -316,12 +327,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -659,7 +672,7 @@
   <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -684,7 +697,7 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
@@ -744,7 +757,7 @@
       <c r="G3" s="3">
         <v>2</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I3" s="3"/>
@@ -772,8 +785,8 @@
       <c r="G4" s="3">
         <v>3</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>12</v>
+      <c r="H4" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3" t="s">
@@ -802,7 +815,7 @@
       <c r="G5" s="3">
         <v>4</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>19</v>
       </c>
       <c r="I5" s="3" t="s">
@@ -832,7 +845,7 @@
       <c r="G6" s="3">
         <v>5</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="4" t="s">
         <v>21</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -862,7 +875,7 @@
       <c r="G7" s="3">
         <v>6</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I7" s="3"/>
@@ -890,7 +903,7 @@
       <c r="G8" s="3">
         <v>7</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="4" t="s">
         <v>21</v>
       </c>
       <c r="I8" s="3" t="s">
@@ -922,7 +935,7 @@
       <c r="G9" s="3">
         <v>8</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I9" s="3"/>
@@ -950,7 +963,7 @@
       <c r="G10" s="3">
         <v>9</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I10" s="3" t="s">
@@ -980,7 +993,7 @@
       <c r="G11" s="3">
         <v>10</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I11" s="3" t="s">
@@ -1012,7 +1025,7 @@
       <c r="G12" s="3">
         <v>11</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="4" t="s">
         <v>21</v>
       </c>
       <c r="I12" s="3" t="s">
@@ -1042,7 +1055,7 @@
       <c r="G13" s="3">
         <v>12</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="4" t="s">
         <v>21</v>
       </c>
       <c r="I13" s="3" t="s">
@@ -1072,7 +1085,7 @@
       <c r="G14" s="3">
         <v>13</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H14" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I14" s="3"/>
@@ -1100,7 +1113,7 @@
       <c r="G15" s="3">
         <v>14</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H15" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I15" s="3" t="s">
@@ -1130,8 +1143,8 @@
       <c r="G16" s="3">
         <v>15</v>
       </c>
-      <c r="H16" s="3" t="s">
-        <v>12</v>
+      <c r="H16" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
@@ -1188,7 +1201,7 @@
       <c r="G18" s="3">
         <v>17</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="H18" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I18" s="3"/>
@@ -1216,7 +1229,7 @@
       <c r="G19" s="3">
         <v>18</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="H19" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I19" s="3"/>
@@ -1244,7 +1257,7 @@
       <c r="G20" s="3">
         <v>19</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H20" s="4" t="s">
         <v>21</v>
       </c>
       <c r="I20" s="3" t="s">
@@ -1274,7 +1287,7 @@
       <c r="G21" s="3">
         <v>20</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="H21" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I21" s="3" t="s">
@@ -1304,7 +1317,7 @@
       <c r="G22" s="3">
         <v>21</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="H22" s="4" t="s">
         <v>21</v>
       </c>
       <c r="I22" s="3" t="s">
@@ -1334,7 +1347,7 @@
       <c r="G23" s="3">
         <v>22</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H23" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I23" s="3"/>
@@ -1362,7 +1375,7 @@
       <c r="G24" s="3">
         <v>23</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="H24" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I24" s="3" t="s">
@@ -1392,7 +1405,7 @@
       <c r="G25" s="3">
         <v>24</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="H25" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I25" s="3" t="s">
@@ -1424,7 +1437,7 @@
       <c r="G26" s="3">
         <v>25</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="H26" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I26" s="3" t="s">
@@ -1456,7 +1469,7 @@
       <c r="G27" s="3">
         <v>26</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="H27" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I27" s="3"/>
@@ -1486,7 +1499,7 @@
       <c r="G28" s="3">
         <v>27</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="H28" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I28" s="3"/>
@@ -1514,8 +1527,8 @@
       <c r="G29" s="3">
         <v>28</v>
       </c>
-      <c r="H29" s="3" t="s">
-        <v>12</v>
+      <c r="H29" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>12</v>
@@ -1546,7 +1559,7 @@
       <c r="G30" s="3">
         <v>29</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="H30" s="4" t="s">
         <v>19</v>
       </c>
       <c r="I30" s="3" t="s">
@@ -1610,7 +1623,7 @@
       <c r="G32" s="3">
         <v>31</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H32" s="4" t="s">
         <v>19</v>
       </c>
       <c r="I32" s="3"/>
@@ -1670,7 +1683,7 @@
       <c r="G34" s="3">
         <v>33</v>
       </c>
-      <c r="H34" s="3" t="s">
+      <c r="H34" s="4" t="s">
         <v>19</v>
       </c>
       <c r="I34" s="3"/>
@@ -1700,7 +1713,7 @@
       <c r="G35" s="3">
         <v>34</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="H35" s="4" t="s">
         <v>19</v>
       </c>
       <c r="I35" s="3" t="s">
@@ -1732,7 +1745,7 @@
       <c r="G36" s="3">
         <v>35</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="H36" s="4" t="s">
         <v>12</v>
       </c>
       <c r="I36" s="3"/>
@@ -1760,7 +1773,7 @@
       <c r="G37" s="3">
         <v>36</v>
       </c>
-      <c r="H37" s="3" t="s">
+      <c r="H37" s="4" t="s">
         <v>21</v>
       </c>
       <c r="I37" s="3" t="s">
@@ -1792,7 +1805,7 @@
       <c r="G38" s="3">
         <v>37</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="H38" s="4" t="s">
         <v>19</v>
       </c>
       <c r="I38" s="3" t="s">
@@ -1824,7 +1837,7 @@
       <c r="G39" s="3">
         <v>38</v>
       </c>
-      <c r="H39" s="3"/>
+      <c r="H39" s="4"/>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
     </row>
@@ -1850,7 +1863,7 @@
       <c r="G40" s="3">
         <v>39</v>
       </c>
-      <c r="H40" s="3"/>
+      <c r="H40" s="4"/>
       <c r="I40" s="3" t="s">
         <v>12</v>
       </c>
@@ -1878,7 +1891,7 @@
       <c r="G41" s="3">
         <v>40</v>
       </c>
-      <c r="H41" s="3"/>
+      <c r="H41" s="4"/>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
     </row>
@@ -1904,7 +1917,7 @@
       <c r="G42" s="3">
         <v>41</v>
       </c>
-      <c r="H42" s="3"/>
+      <c r="H42" s="4"/>
       <c r="I42" s="3"/>
     </row>
   </sheetData>

</xml_diff>